<commit_message>
Update ESS power-limit classification, carbon accounting, and Figure 4 outputs
</commit_message>
<xml_diff>
--- a/Figure_Plot/figure_plot_4_a_b/source_data/dsfunction_May2025_exact_V5_k20_classified.xlsx
+++ b/Figure_Plot/figure_plot_4_a_b/source_data/dsfunction_May2025_exact_V5_k20_classified.xlsx
@@ -15988,7 +15988,7 @@
       </c>
       <c r="F598" s="4" t="inlineStr">
         <is>
-          <t>[0,16.6315309082,1.750687464,0,1.313015598]</t>
+          <t>[0,0,1.750687464,0,1.313015598]</t>
         </is>
       </c>
     </row>
@@ -16014,7 +16014,7 @@
       </c>
       <c r="F599" s="4" t="inlineStr">
         <is>
-          <t>[0,16.7827991083,1.3607674953,0,1.8143566604]</t>
+          <t>[0,0,1.3607674953,0,1.8143566604]</t>
         </is>
       </c>
     </row>
@@ -16040,7 +16040,7 @@
       </c>
       <c r="F600" s="4" t="inlineStr">
         <is>
-          <t>[0,17.8011135412,1.3693164262,0,1.825755235]</t>
+          <t>[0,0,1.3693164262,0,1.825755235]</t>
         </is>
       </c>
     </row>
@@ -16066,7 +16066,7 @@
       </c>
       <c r="F601" s="4" t="inlineStr">
         <is>
-          <t>[0,16.8011129209,1.4400953932,0,1.4400953932]</t>
+          <t>[0,0,1.4400953932,0,1.4400953932]</t>
         </is>
       </c>
     </row>
@@ -16092,7 +16092,7 @@
       </c>
       <c r="F602" s="4" t="inlineStr">
         <is>
-          <t>[0,17.0457152914,1.4204762743,0,1.8939683657]</t>
+          <t>[0,0,1.4204762743,0,1.8939683657]</t>
         </is>
       </c>
     </row>
@@ -16118,7 +16118,7 @@
       </c>
       <c r="F603" s="4" t="inlineStr">
         <is>
-          <t>[0,16.8625319601,1.4453598823,0,1.4453598823]</t>
+          <t>[0,0,1.4453598823,0,1.4453598823]</t>
         </is>
       </c>
     </row>
@@ -16144,7 +16144,7 @@
       </c>
       <c r="F604" s="4" t="inlineStr">
         <is>
-          <t>[0,16.9755098227,1.4146258186,0,1.4146258186]</t>
+          <t>[0,0,1.4146258186,0,1.4146258186]</t>
         </is>
       </c>
     </row>
@@ -16162,7 +16162,7 @@
       </c>
       <c r="D605" s="4" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E605" t="n">
@@ -16170,7 +16170,7 @@
       </c>
       <c r="F605" s="4" t="inlineStr">
         <is>
-          <t>[0,20.4297334611,1.9456889011,0,0]</t>
+          <t>[0,0,1.9456889011,0,0]</t>
         </is>
       </c>
     </row>

</xml_diff>